<commit_message>
chore: compress large social videos and retry push
</commit_message>
<xml_diff>
--- a/public/website products/Updated pricelist 12.03.26 - Copy.xlsx
+++ b/public/website products/Updated pricelist 12.03.26 - Copy.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Desktop/out of box web /public/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Desktop/out of box web /public/website products/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED628764-F4DD-C74C-886B-19E045888201}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{860FA65C-124F-5141-84C3-91B97982519B}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="40" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="25300" activeTab="1" xr2:uid="{44EC185D-A192-4C91-92C2-82238AE89C8A}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26380" firstSheet="1" activeTab="1" xr2:uid="{44EC185D-A192-4C91-92C2-82238AE89C8A}"/>
   </bookViews>
   <sheets>
     <sheet name="QuickBooks Export Tips" sheetId="2" r:id="rId1"/>
@@ -4276,7 +4276,7 @@
     <t>Starting Price (VAT Incl)</t>
   </si>
   <si>
-    <t xml:space="preserve">PRODUCT NAME </t>
+    <t>PRODUCT NAME</t>
   </si>
 </sst>
 </file>
@@ -4317,6 +4317,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -4498,7 +4499,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>520700</xdr:colOff>
+          <xdr:colOff>495300</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
@@ -4560,7 +4561,7 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>520700</xdr:colOff>
+          <xdr:colOff>495300</xdr:colOff>
           <xdr:row>0</xdr:row>
           <xdr:rowOff>228600</xdr:rowOff>
         </xdr:to>
@@ -5752,20 +5753,20 @@
     <row r="2" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" ht="25.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" ht="21" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="6" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="8" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="9" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="10" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="11" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="12" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="13" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="14" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="15" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="16" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="17" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="18" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="19" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="7" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="9" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="10" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="14" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="15" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="17" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B40" s="7"/>
       <c r="C40" s="7"/>
@@ -14386,7 +14387,7 @@
         <v>858</v>
       </c>
       <c r="D860" s="9">
-        <v>3500</v>
+        <v>3100</v>
       </c>
     </row>
     <row r="861" spans="1:4" x14ac:dyDescent="0.2">
@@ -15026,7 +15027,7 @@
         <v>922</v>
       </c>
       <c r="D924" s="9">
-        <v>15015.00000088</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="925" spans="1:4" x14ac:dyDescent="0.2">
@@ -15236,7 +15237,7 @@
         <v>943</v>
       </c>
       <c r="D945" s="9">
-        <v>8000</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="946" spans="1:4" x14ac:dyDescent="0.2">
@@ -15626,7 +15627,7 @@
       </c>
       <c r="C984" s="2"/>
       <c r="D984" s="9">
-        <v>3749716.2997580003</v>
+        <v>3750816.2997690002</v>
       </c>
     </row>
     <row r="985" spans="1:4" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.15">
@@ -15636,7 +15637,7 @@
       <c r="B985" s="1"/>
       <c r="C985" s="1"/>
       <c r="D985" s="9">
-        <v>3749716.2997580003</v>
+        <v>3750816.2997690002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>